<commit_message>
Cập nhật tài khoản: 16/09/2026 17:49
</commit_message>
<xml_diff>
--- a/config/Config_Users.xlsx
+++ b/config/Config_Users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhuan\Desktop\portal_nuoc_sach_sonla-main\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63C0DCC8-6A15-4E04-943B-444297DA8D83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFCC97B-058A-4215-8C3A-33318DDF08D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
   <si>
     <t>STT</t>
   </si>
@@ -83,6 +83,12 @@
   </si>
   <si>
     <t>phiengkhoai</t>
+  </si>
+  <si>
+    <t>Xã Phiêng Cằm</t>
+  </si>
+  <si>
+    <t>phiengcam</t>
   </si>
 </sst>
 </file>
@@ -422,7 +428,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="5" width="20" customWidth="1"/>
@@ -564,6 +570,23 @@
         <v>7</v>
       </c>
     </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" t="s">
+        <v>7</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cập nhật tài khoản: 16/09/2026 18:05
</commit_message>
<xml_diff>
--- a/config/Config_Users.xlsx
+++ b/config/Config_Users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhuan\Desktop\portal_nuoc_sach_sonla-main\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEFCC97B-058A-4215-8C3A-33318DDF08D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56938302-74EB-413C-8F89-8B1F19ECE5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="24">
   <si>
     <t>STT</t>
   </si>
@@ -34,18 +34,12 @@
     <t>Mat_Khau</t>
   </si>
   <si>
-    <t>Khoa</t>
-  </si>
-  <si>
     <t>ADMIN</t>
   </si>
   <si>
     <t>admin</t>
   </si>
   <si>
-    <t>Không</t>
-  </si>
-  <si>
     <t>Xã Tân Lập</t>
   </si>
   <si>
@@ -89,6 +83,15 @@
   </si>
   <si>
     <t>phiengcam</t>
+  </si>
+  <si>
+    <t>Vaitro</t>
+  </si>
+  <si>
+    <t>Quản trị</t>
+  </si>
+  <si>
+    <t>Các xã/phường</t>
   </si>
 </sst>
 </file>
@@ -448,7 +451,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -456,16 +459,16 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E2" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -473,16 +476,16 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -490,16 +493,16 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -507,16 +510,16 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -524,16 +527,16 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -541,16 +544,16 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -558,16 +561,16 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D8" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -575,16 +578,16 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>7</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cập nhật tài khoản: 16/09/2026 18:17
</commit_message>
<xml_diff>
--- a/config/Config_Users.xlsx
+++ b/config/Config_Users.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nhuan\Desktop\portal_nuoc_sach_sonla-main\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F668A432-5C5D-49E2-B171-60C8A74281B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6121ECCE-B0E9-44E3-AA9E-070C456A2C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -88,10 +88,10 @@
     <t>Quản trị</t>
   </si>
   <si>
-    <t>Các xã/phường</t>
-  </si>
-  <si>
     <t>Khoa</t>
+  </si>
+  <si>
+    <t>Tài khoản xã/phường</t>
   </si>
 </sst>
 </file>
@@ -434,7 +434,8 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="20" customWidth="1"/>
+    <col min="1" max="1" width="4.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -451,7 +452,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -485,7 +486,7 @@
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -502,7 +503,7 @@
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -519,7 +520,7 @@
         <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -536,7 +537,7 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -553,7 +554,7 @@
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -570,7 +571,7 @@
         <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -587,7 +588,7 @@
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>